<commit_message>
feat: sincroniza modulos recentes (saida osme, contagem carro/deposito, atualizar osme, tray e updater online)
</commit_message>
<xml_diff>
--- a/data/banco_de_dados.xlsx
+++ b/data/banco_de_dados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anderson.vieira\Desktop\DEV\PROJETO MODULAR 2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F12F8F-D07C-4B69-A882-9AA923D70A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA528F2-9917-4266-8F5A-180B8AE6969A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8565" yWindow="6165" windowWidth="15000" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PASTA1" sheetId="3" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="114">
   <si>
     <t>Material</t>
   </si>
@@ -389,6 +389,18 @@
   </si>
   <si>
     <t>CAIXA,POLIC,MED BIFASICO,LENTE</t>
+  </si>
+  <si>
+    <t>MED. ELETR.15-120A,120V,3E,4F- 199.59</t>
+  </si>
+  <si>
+    <t>MED.ELETR.2,5/5 -10/20A,120/240V,3E4F</t>
+  </si>
+  <si>
+    <t>MED. ELETR.15-120A,120/240V,3E,4F-CENTR</t>
+  </si>
+  <si>
+    <t>MED. ELETR.15-120A,120V,3E,4F-GD 199.59</t>
   </si>
 </sst>
 </file>
@@ -1760,20 +1772,48 @@
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
+      <c r="A89" s="2">
+        <v>510905</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90" s="2"/>
-      <c r="B90" s="2"/>
+      <c r="A90" s="2">
+        <v>510848</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
+      <c r="A91" s="2">
+        <v>510850</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
+      <c r="A92" s="2">
+        <v>510903</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>

</xml_diff>

<commit_message>
feat(v2.3.2): atualizacao completa N.E.X.U.S v2.3.2 - higienizacao de seriais, motor updater zero-lock e melhorias de UI/resiliencia
</commit_message>
<xml_diff>
--- a/data/banco_de_dados.xlsx
+++ b/data/banco_de_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anderson.vieira\Desktop\DEV\PROJETO MODULAR 2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA528F2-9917-4266-8F5A-180B8AE6969A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6232653E-6F8D-44E0-AA94-0D4C14BB24E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8565" yWindow="6165" windowWidth="15000" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PASTA1" sheetId="3" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="115">
   <si>
     <t>Material</t>
   </si>
@@ -401,6 +401,9 @@
   </si>
   <si>
     <t>MED. ELETR.15-120A,120V,3E,4F-GD 199.59</t>
+  </si>
+  <si>
+    <t>CABO,AEREO,AL,MULT,2X1X10+ 10,GSCC09/20</t>
   </si>
 </sst>
 </file>
@@ -1816,8 +1819,15 @@
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A93" s="2"/>
-      <c r="B93" s="2"/>
+      <c r="A93" s="2">
+        <v>324062</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>

</xml_diff>